<commit_message>
continue candidate mass upload
</commit_message>
<xml_diff>
--- a/JobOfferSolution/JO.BlazorApp/wwwroot/template/candidate-massupload.xlsx
+++ b/JobOfferSolution/JO.BlazorApp/wwwroot/template/candidate-massupload.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\JobOfferSolution\JO.BlazorApp\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3E824E7-A295-491C-93E8-AB5FEF5DE3D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BEF325-0D3E-4E49-B901-832F4EB2A34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25104" yWindow="3636" windowWidth="17160" windowHeight="7836" xr2:uid="{09AD2D92-39CA-4F02-AC5C-5575F6ABAA7C}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09AD2D92-39CA-4F02-AC5C-5575F6ABAA7C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>FirstName</t>
   </si>
@@ -53,28 +53,19 @@
     <t>Email</t>
   </si>
   <si>
-    <t>MobileNumber</t>
-  </si>
-  <si>
     <t>PositionApplied</t>
   </si>
   <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>HiringManager</t>
-  </si>
-  <si>
-    <t>Recruiter</t>
+    <t>CompanyCode</t>
+  </si>
+  <si>
+    <t>ContactNumber</t>
+  </si>
+  <si>
+    <t>DivisionCode</t>
   </si>
   <si>
     <t>ExpectedSalary</t>
-  </si>
-  <si>
-    <t>StartDate</t>
-  </si>
-  <si>
-    <t>Remarks</t>
   </si>
 </sst>
 </file>
@@ -446,24 +437,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{675211B3-3D98-4A62-B5E8-901970671D19}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -477,28 +467,19 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
       </c>
       <c r="H1" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>